<commit_message>
Add final demo data set, script, rehearsal transcripts and video edit tooling
- Set F demo data (seed-data/demo-final): 25 accounts, 11 contacts, 2 history
  projects, 5 won opportunities, 8 parties, email and call activities, the
  Dodge W40 spreadsheet; seeded with clio and listed in the fixture manifest
- Excel fix: Dodge IDs without long digit runs (the PII phone detector
  masked the old IDs, so every row was blocked)
- FINAL-demo-script.md: 4-minute script (workspace, scoring, chat, Excel,
  email) with prompts, expected answers and voice-over; script 09 moved to Set F
- Rehearsal transcripts of the 29 Sep test chats and the implementation log
- Video tooling: GIF-to-WebM converter, 14-min edit and silent 5-min cut
  scripts, timed voice-over (md, srt, json). Video files stay local (*.mp4
  ignored)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed-data/demo/Dodge_Weekly_Export_2026-09-29.xlsx
+++ b/seed-data/demo/Dodge_Weekly_Export_2026-09-29.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DG-26-114872</t>
+          <t>DG-PT4872</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DG-26-115390</t>
+          <t>DG-BH5390</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DG-26-116004</t>
+          <t>DG-BC6004</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>